<commit_message>
Cargados IDPAC y Esteban
</commit_message>
<xml_diff>
--- a/originales/respuestas/2025/01. Calificadas/bucle p1/Secretaría Distrital De Desarrollo Económico.xlsx
+++ b/originales/respuestas/2025/01. Calificadas/bucle p1/Secretaría Distrital De Desarrollo Económico.xlsx
@@ -1521,7 +1521,11 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="29" width="10.71"/>
+    <col customWidth="1" min="1" max="3" width="10.71"/>
+    <col customWidth="1" min="4" max="4" width="47.43"/>
+    <col customWidth="1" min="5" max="5" width="24.57"/>
+    <col customWidth="1" min="6" max="7" width="25.57"/>
+    <col customWidth="1" min="8" max="29" width="10.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="43.5" customHeight="1">

</xml_diff>